<commit_message>
Daily NAV update 2026-03-11
</commit_message>
<xml_diff>
--- a/output/nav_changes_2026-03-11.xlsx
+++ b/output/nav_changes_2026-03-11.xlsx
@@ -801,16 +801,16 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>20.21</v>
+        <v>20.205</v>
       </c>
       <c r="E11" s="6" t="n">
         <v>20.22</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>-0.01</v>
+        <v>-0.015</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>-0.0495</v>
+        <v>-0.0742</v>
       </c>
     </row>
     <row r="12">
@@ -821,33 +821,25 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0P0000MOQB.TO</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>14.2968</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>14.2588</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>0.2665</v>
       </c>
     </row>
     <row r="13">
@@ -948,7 +940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -964,6 +956,7 @@
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1032,11 +1025,16 @@
           <t>Dynamic Short Term Credit PLUS F</t>
         </is>
       </c>
+      <c r="N1" s="9" t="inlineStr">
+        <is>
+          <t>Pender Corporate Bond F</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -1044,1690 +1042,1762 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" s="7" t="n">
-        <v>0.0274</v>
+      <c r="E2" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="5" t="n">
-        <v>-0.5536</v>
+      <c r="H2" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>-0.0495</v>
-      </c>
-      <c r="J2" s="5" t="n">
-        <v>-0.185</v>
+        <v>-0.0247</v>
+      </c>
+      <c r="J2" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" s="5" t="n">
-        <v>-0.149</v>
-      </c>
+      <c r="M2" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>-0.2505</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>-0.1991</v>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>0.1388</v>
-      </c>
-      <c r="E3" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="7" t="n">
-        <v>0.0369</v>
-      </c>
-      <c r="G3" s="5" t="n">
-        <v>-0.0499</v>
-      </c>
-      <c r="H3" s="7" t="n">
-        <v>0.5058</v>
-      </c>
-      <c r="I3" s="7" t="n">
-        <v>0.1982</v>
-      </c>
-      <c r="J3" s="7" t="n">
-        <v>0.1854</v>
-      </c>
-      <c r="K3" s="5" t="n">
-        <v>-0.1102</v>
-      </c>
-      <c r="L3" s="7" t="n">
-        <v>0.0978</v>
-      </c>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" s="7" t="n">
+        <v>0.0274</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" s="5" t="n">
+        <v>-0.5536</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>-0.0495</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>-0.185</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" s="5" t="n">
-        <v>-0.0992</v>
-      </c>
+        <v>-0.149</v>
+      </c>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="n">
-        <v>0</v>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>-0.2505</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>-0.3561</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>-0.3548</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>-0.3274</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>-0.2123</v>
+        <v>-0.1991</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>0.1388</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>0.0369</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>-0.1462</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>-0.403</v>
-      </c>
-      <c r="I4" s="5" t="n">
-        <v>-0.3457</v>
-      </c>
-      <c r="J4" s="5" t="n">
-        <v>-0.2773</v>
+        <v>-0.0499</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>0.5058</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>0.1982</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>0.1854</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>-0.3356</v>
-      </c>
-      <c r="L4" s="5" t="n">
-        <v>-0.2977</v>
-      </c>
-      <c r="M4" s="10" t="n">
-        <v>0</v>
-      </c>
+        <v>-0.1102</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>0.0978</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>-0.0992</v>
+      </c>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="n">
-        <v>0.0501</v>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>-0.2536</v>
+        <v>-0.3561</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>-0.3648</v>
+        <v>-0.3548</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>-0.0273</v>
+        <v>-0.3274</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>-0.3766</v>
+        <v>-0.2123</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>-0.172</v>
+        <v>-0.1462</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>-0.3514</v>
+        <v>-0.403</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.4425</v>
+        <v>-0.3457</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>-0.3683</v>
+        <v>-0.2773</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>-0.2056</v>
+        <v>-0.3356</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>-0.2675</v>
+        <v>-0.2977</v>
       </c>
       <c r="M5" s="10" t="n">
         <v>0</v>
       </c>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>0.1008</v>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.0501</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>-0.2536</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>-0.0169</v>
+        <v>-0.3648</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>-0.2177</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>0.0443</v>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>0.0068</v>
-      </c>
-      <c r="H6" s="7" t="n">
-        <v>0.1005</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>0.0984</v>
-      </c>
-      <c r="J6" s="7" t="n">
-        <v>0.0922</v>
-      </c>
-      <c r="K6" s="7" t="n">
-        <v>0.1065</v>
-      </c>
-      <c r="L6" s="7" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="M6" s="7" t="n">
-        <v>0.0993</v>
-      </c>
+        <v>-0.0273</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>-0.3766</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>-0.172</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>-0.3514</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>-0.4425</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>-0.3683</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>-0.2056</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>-0.2675</v>
+      </c>
+      <c r="M6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>-0.1498</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>-0.4026</v>
+        <v>-0.25</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>0.1008</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>-0.1943</v>
+        <v>-0.0169</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>-0.3256</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>-0.3679</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>-0.2089</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>-0.0502</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>-0.1474</v>
-      </c>
-      <c r="J7" s="5" t="n">
-        <v>-0.1381</v>
-      </c>
-      <c r="K7" s="5" t="n">
-        <v>-0.5051</v>
-      </c>
-      <c r="L7" s="5" t="n">
-        <v>-0.2377</v>
-      </c>
-      <c r="M7" s="5" t="n">
-        <v>-0.2476</v>
-      </c>
+        <v>-0.2177</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>0.0443</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>0.1005</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>0.0984</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>0.0922</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>0.1065</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>0.0537</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>0.0993</v>
+      </c>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>-0.0499</v>
+        <v>-0.1498</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>-0.2881</v>
+        <v>-0.4026</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>-0.362</v>
+        <v>-0.1943</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>-0.2166</v>
+        <v>-0.3256</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>-0.3655</v>
+        <v>-0.3679</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>-0.2646</v>
+        <v>-0.2089</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>-0.4002</v>
+        <v>-0.0502</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>-0.489</v>
+        <v>-0.1474</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>-0.3668</v>
-      </c>
-      <c r="K8" s="7" t="n">
-        <v>0.2396</v>
+        <v>-0.1381</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>-0.5051</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>-0.3236</v>
+        <v>-0.2377</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>-0.3455</v>
-      </c>
+        <v>-0.2476</v>
+      </c>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="n">
-        <v>0</v>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>-0.0499</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>-0.0413</v>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>0.0958</v>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>0.217</v>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>0.0418</v>
-      </c>
-      <c r="G9" s="7" t="n">
-        <v>0.0225</v>
-      </c>
-      <c r="H9" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="7" t="n">
-        <v>0.0979</v>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>0.0459</v>
+        <v>-0.2881</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>-0.362</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>-0.2166</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>-0.3655</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>-0.2646</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>-0.4002</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>-0.489</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>-0.3668</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>0.1012</v>
-      </c>
-      <c r="L9" s="7" t="n">
-        <v>0.005</v>
+        <v>0.2396</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>-0.3236</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>-0.197</v>
-      </c>
+        <v>-0.3455</v>
+      </c>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="n">
-        <v>0.07489999999999999</v>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>0.0483</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>-0.0357</v>
-      </c>
-      <c r="E10" s="10" t="n">
-        <v>0</v>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>-0.0413</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>0.0958</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>0.217</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>0.2752</v>
+        <v>0.0418</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>0.0011</v>
+        <v>0.0225</v>
       </c>
       <c r="H10" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>0.049</v>
+        <v>0.0979</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>0.09180000000000001</v>
-      </c>
-      <c r="K10" s="5" t="n">
-        <v>-0.099</v>
+        <v>0.0459</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>0.1012</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>0.0757</v>
-      </c>
-      <c r="M10" s="7" t="n">
-        <v>0.09859999999999999</v>
-      </c>
+        <v>0.005</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>-0.197</v>
+      </c>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>-0.025</v>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0.07489999999999999</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>0.0105</v>
+        <v>0.0483</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>-0.0803</v>
+        <v>-0.0357</v>
       </c>
       <c r="E11" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="5" t="n">
-        <v>-0.09130000000000001</v>
+      <c r="F11" s="7" t="n">
+        <v>0.2752</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>0.007900000000000001</v>
+        <v>0.0011</v>
       </c>
       <c r="H11" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="5" t="n">
-        <v>-0.0489</v>
-      </c>
-      <c r="J11" s="5" t="n">
-        <v>-0.0917</v>
-      </c>
-      <c r="K11" s="7" t="n">
-        <v>0.0552</v>
-      </c>
-      <c r="L11" s="5" t="n">
-        <v>-0.0202</v>
-      </c>
-      <c r="M11" s="5" t="n">
-        <v>-0.0985</v>
-      </c>
+      <c r="I11" s="7" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>0.09180000000000001</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>-0.099</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>0.0757</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>0.09859999999999999</v>
+      </c>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>0.125</v>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>-0.025</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>0.0299</v>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>0.0308</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>-0.0813</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>0.06560000000000001</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>-0.0439</v>
-      </c>
-      <c r="H12" s="5" t="n">
-        <v>-0.01</v>
+        <v>0.0105</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>-0.0803</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>-0.09130000000000001</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>0.007900000000000001</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-0.0978</v>
+        <v>-0.0489</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>-0.0229</v>
-      </c>
-      <c r="K12" s="5" t="n">
-        <v>-0.0052</v>
-      </c>
-      <c r="L12" s="7" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="M12" s="7" t="n">
-        <v>0.0246</v>
-      </c>
+        <v>-0.0917</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>0.0552</v>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>-0.0202</v>
+      </c>
+      <c r="M12" s="5" t="n">
+        <v>-0.0985</v>
+      </c>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="n">
-        <v>0</v>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>0.125</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>0.1038</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>-0.0698</v>
-      </c>
-      <c r="E13" s="7" t="n">
-        <v>0.2991</v>
+        <v>0.0299</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0.0308</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>-0.0813</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>0.1442</v>
-      </c>
-      <c r="G13" s="7" t="n">
-        <v>0.1477</v>
-      </c>
-      <c r="H13" s="7" t="n">
-        <v>0.09959999999999999</v>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>0.0974</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>0.1373</v>
+        <v>0.06560000000000001</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>-0.0439</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>-0.0978</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>-0.0229</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>-0.18</v>
+        <v>-0.0052</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>0.098</v>
-      </c>
-      <c r="M13" s="5" t="n">
-        <v>-0.0492</v>
-      </c>
+        <v>0.004</v>
+      </c>
+      <c r="M13" s="7" t="n">
+        <v>0.0246</v>
+      </c>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>-0.05</v>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>0.0466</v>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>0.0196</v>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>-0.2062</v>
+        <v>0.1038</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>-0.0698</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0.2991</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>0.0528</v>
-      </c>
-      <c r="G14" s="5" t="n">
-        <v>-0.0045</v>
-      </c>
-      <c r="H14" s="5" t="n">
-        <v>-0.0495</v>
+        <v>0.1442</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>0.1477</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>0.09959999999999999</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>0.049</v>
-      </c>
-      <c r="J14" s="10" t="n">
-        <v>0</v>
+        <v>0.0974</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>0.1373</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>-0.2574</v>
+        <v>-0.18</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>0.0445</v>
-      </c>
-      <c r="M14" s="10" t="n">
-        <v>0</v>
-      </c>
+        <v>0.098</v>
+      </c>
+      <c r="M14" s="5" t="n">
+        <v>-0.0492</v>
+      </c>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>-0.0185</v>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>-0.0935</v>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>0.0466</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0.0196</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>-0.0808</v>
+        <v>-0.2062</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>0.0399</v>
-      </c>
-      <c r="G15" s="7" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="H15" s="7" t="n">
-        <v>0.0997</v>
-      </c>
-      <c r="I15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>0.0459</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>0.0914</v>
+        <v>0.0528</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>-0.0045</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>-0.0495</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="J15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>-0.2574</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="M15" s="7" t="n">
-        <v>0.0493</v>
-      </c>
+        <v>0.0445</v>
+      </c>
+      <c r="M15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n">
-        <v>0.05</v>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>-0.0273</v>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>0.0175</v>
+        <v>-0.0185</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>-0.0935</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>-0.0542</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>-0.0409</v>
+        <v>-0.0808</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>0.0399</v>
       </c>
       <c r="G16" s="7" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>0.0997</v>
+      </c>
+      <c r="I16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>0.0459</v>
+      </c>
+      <c r="K16" s="7" t="n">
         <v>0.0914</v>
       </c>
-      <c r="H16" s="5" t="n">
-        <v>-0.1496</v>
-      </c>
-      <c r="I16" s="7" t="n">
-        <v>0.0975</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>0.0225</v>
-      </c>
-      <c r="K16" s="7" t="n">
-        <v>0.0915</v>
-      </c>
       <c r="L16" s="7" t="n">
-        <v>0.0283</v>
-      </c>
-      <c r="M16" s="5" t="n">
-        <v>-0.0492</v>
-      </c>
+        <v>0.001</v>
+      </c>
+      <c r="M16" s="7" t="n">
+        <v>0.0493</v>
+      </c>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>-0.05</v>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>0.1083</v>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>-0.0273</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>0.0922</v>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>0.1351</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>0.11</v>
+        <v>0.0175</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>-0.0542</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>-0.0409</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>0.0339</v>
-      </c>
-      <c r="H17" s="7" t="n">
-        <v>0.1498</v>
-      </c>
-      <c r="I17" s="5" t="n">
-        <v>-0.0975</v>
+        <v>0.0914</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>-0.1496</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>0.0975</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.06900000000000001</v>
-      </c>
-      <c r="K17" s="5" t="n">
-        <v>-0.0031</v>
+        <v>0.0225</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>0.0915</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>0.0779</v>
+        <v>0.0283</v>
       </c>
       <c r="M17" s="5" t="n">
-        <v>-0.0487</v>
-      </c>
+        <v>-0.0492</v>
+      </c>
+      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>0.05</v>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>-0.05</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>0.1579</v>
+        <v>0.1083</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>0.1245</v>
+        <v>0.0922</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>0.217</v>
+        <v>0.1351</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>0.1566</v>
+        <v>0.11</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>0.1051</v>
+        <v>0.0339</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>0.2501</v>
-      </c>
-      <c r="I18" s="7" t="n">
-        <v>0.1958</v>
+        <v>0.1498</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>-0.0975</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>0.0916</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>-0.0114</v>
+        <v>-0.0031</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>0.1012</v>
-      </c>
-      <c r="M18" s="7" t="n">
-        <v>0.1474</v>
-      </c>
+        <v>0.0779</v>
+      </c>
+      <c r="M18" s="5" t="n">
+        <v>-0.0487</v>
+      </c>
+      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>0.09959999999999999</v>
+        <v>0.05</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>0.2042</v>
+        <v>0.1579</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>0.1499</v>
+        <v>0.1245</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.1896</v>
+        <v>0.217</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>0.2729</v>
+        <v>0.1566</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>0.2834</v>
+        <v>0.1051</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.5032</v>
+        <v>0.2501</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.245</v>
+        <v>0.1958</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.1609</v>
+        <v>0.0916</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>-0.0644</v>
+        <v>-0.0114</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>0.2059</v>
-      </c>
-      <c r="M19" s="5" t="n">
-        <v>-0.1472</v>
-      </c>
+        <v>0.1012</v>
+      </c>
+      <c r="M19" s="7" t="n">
+        <v>0.1474</v>
+      </c>
+      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="n">
-        <v>0</v>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>0.09959999999999999</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>0.1026</v>
+        <v>0.2042</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>0.0575</v>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>-0.0267</v>
-      </c>
-      <c r="F20" s="5" t="n">
-        <v>-0.013</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>-0.0578</v>
-      </c>
-      <c r="H20" s="5" t="n">
-        <v>-0.1507</v>
+        <v>0.1499</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>0.1896</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>0.2729</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>0.2834</v>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>0.5032</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>0.0492</v>
+        <v>0.245</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>0.0692</v>
-      </c>
-      <c r="K20" s="7" t="n">
-        <v>0.0863</v>
+        <v>0.1609</v>
+      </c>
+      <c r="K20" s="5" t="n">
+        <v>-0.0644</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>0.0365</v>
-      </c>
-      <c r="M20" s="7" t="n">
-        <v>0.1227</v>
-      </c>
+        <v>0.2059</v>
+      </c>
+      <c r="M20" s="5" t="n">
+        <v>-0.1472</v>
+      </c>
+      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="n">
-        <v>0.1002</v>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>0.1347</v>
+        <v>0.1026</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>0.1327</v>
-      </c>
-      <c r="E21" s="7" t="n">
-        <v>0.054</v>
-      </c>
-      <c r="F21" s="7" t="n">
-        <v>0.2638</v>
-      </c>
-      <c r="G21" s="7" t="n">
-        <v>0.1055</v>
-      </c>
-      <c r="H21" s="7" t="n">
-        <v>0.3023</v>
+        <v>0.0575</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>-0.0267</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>-0.013</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>-0.0578</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>-0.1507</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.0487</v>
+        <v>0.0492</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.0919</v>
+        <v>0.0692</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>0.1353</v>
+        <v>0.0863</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>0.1219</v>
+        <v>0.0365</v>
       </c>
       <c r="M21" s="7" t="n">
-        <v>0.0246</v>
-      </c>
+        <v>0.1227</v>
+      </c>
+      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="n">
-        <v>0</v>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>0.1002</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>0.0683</v>
+        <v>0.1347</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>0.0239</v>
+        <v>0.1327</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>0.1632</v>
+        <v>0.054</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>0.0163</v>
+        <v>0.2638</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>0.0113</v>
-      </c>
-      <c r="H22" s="5" t="n">
-        <v>-0.0505</v>
+        <v>0.1055</v>
+      </c>
+      <c r="H22" s="7" t="n">
+        <v>0.3023</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>0.0493</v>
+        <v>0.0487</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>0.0462</v>
-      </c>
-      <c r="K22" s="5" t="n">
-        <v>-0.4282</v>
-      </c>
-      <c r="L22" s="5" t="n">
-        <v>-0.0163</v>
+        <v>0.0919</v>
+      </c>
+      <c r="K22" s="7" t="n">
+        <v>0.1353</v>
+      </c>
+      <c r="L22" s="7" t="n">
+        <v>0.1219</v>
       </c>
       <c r="M22" s="7" t="n">
-        <v>0.1471</v>
-      </c>
+        <v>0.0246</v>
+      </c>
+      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="n">
-        <v>0.0998</v>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>0.0364</v>
+        <v>0.0683</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>0.0513</v>
+        <v>0.0239</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.1635</v>
+        <v>0.1632</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>0.0511</v>
+        <v>0.0163</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>0.0499</v>
-      </c>
-      <c r="H23" s="7" t="n">
-        <v>0.0505</v>
+        <v>0.0113</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>-0.0505</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.09810000000000001</v>
+        <v>0.0493</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.0458</v>
+        <v>0.0462</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>-0.2038</v>
-      </c>
-      <c r="L23" s="7" t="n">
-        <v>0.0163</v>
-      </c>
-      <c r="M23" s="10" t="n">
-        <v>0</v>
-      </c>
+        <v>-0.4282</v>
+      </c>
+      <c r="L23" s="5" t="n">
+        <v>-0.0163</v>
+      </c>
+      <c r="M23" s="7" t="n">
+        <v>0.1471</v>
+      </c>
+      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>-0.1497</v>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>0.0998</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>0.09229999999999999</v>
+        <v>0.0364</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>0.0316</v>
+        <v>0.0513</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>0.0273</v>
+        <v>0.1635</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>0.197</v>
+        <v>0.0511</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>0.06469999999999999</v>
+        <v>0.0499</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>0.4555</v>
+        <v>0.0505</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>0.0493</v>
+        <v>0.09810000000000001</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>0.2772</v>
+        <v>0.0458</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>-0.08790000000000001</v>
+        <v>-0.2038</v>
       </c>
       <c r="L24" s="7" t="n">
-        <v>0.1058</v>
+        <v>0.0163</v>
       </c>
       <c r="M24" s="10" t="n">
         <v>0</v>
       </c>
+      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="n">
-        <v>0.1002</v>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>-0.047</v>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>-0.1497</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>0.09229999999999999</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>0.0183</v>
-      </c>
-      <c r="E25" s="5" t="n">
-        <v>-0.0273</v>
+        <v>0.0316</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>0.0273</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>0.0044</v>
+        <v>0.197</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>0.0432</v>
-      </c>
-      <c r="H25" s="5" t="n">
-        <v>-0.1009</v>
+        <v>0.06469999999999999</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>0.4555</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.0494</v>
-      </c>
-      <c r="J25" s="5" t="n">
-        <v>-0.1384</v>
-      </c>
-      <c r="K25" s="7" t="n">
-        <v>0.06619999999999999</v>
+        <v>0.0493</v>
+      </c>
+      <c r="J25" s="7" t="n">
+        <v>0.2772</v>
+      </c>
+      <c r="K25" s="5" t="n">
+        <v>-0.08790000000000001</v>
       </c>
       <c r="L25" s="7" t="n">
-        <v>0.0122</v>
-      </c>
-      <c r="M25" s="7" t="n">
-        <v>0.0494</v>
-      </c>
+        <v>0.1058</v>
+      </c>
+      <c r="M25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n">
-        <v>-0.0501</v>
-      </c>
-      <c r="C26" s="7" t="n">
-        <v>0.0257</v>
-      </c>
-      <c r="D26" s="5" t="n">
-        <v>-0.0091</v>
-      </c>
-      <c r="E26" s="7" t="n">
-        <v>0.08210000000000001</v>
-      </c>
-      <c r="F26" s="5" t="n">
-        <v>-0.0011</v>
-      </c>
-      <c r="G26" s="5" t="n">
-        <v>-0.0204</v>
-      </c>
-      <c r="H26" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="10" t="n">
-        <v>0</v>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>0.1002</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>-0.047</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>0.0183</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>-0.0273</v>
+      </c>
+      <c r="F26" s="7" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>0.0432</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>-0.1009</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>0.0494</v>
+      </c>
+      <c r="J26" s="5" t="n">
+        <v>-0.1384</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>0.059</v>
-      </c>
-      <c r="L26" s="5" t="n">
-        <v>-0.0122</v>
-      </c>
-      <c r="M26" s="5" t="n">
-        <v>-0.0494</v>
-      </c>
+        <v>0.06619999999999999</v>
+      </c>
+      <c r="L26" s="7" t="n">
+        <v>0.0122</v>
+      </c>
+      <c r="M26" s="7" t="n">
+        <v>0.0494</v>
+      </c>
+      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="n">
-        <v>0.0501</v>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>-0.0501</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>0.1244</v>
+        <v>0.0257</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>-0.0063</v>
-      </c>
-      <c r="E27" s="5" t="n">
-        <v>-0.1361</v>
+        <v>-0.0091</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>0.08210000000000001</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>-0.0924</v>
-      </c>
-      <c r="G27" s="7" t="n">
-        <v>0.0591</v>
-      </c>
-      <c r="H27" s="5" t="n">
-        <v>-0.1014</v>
+        <v>-0.0011</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>-0.0204</v>
+      </c>
+      <c r="H27" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="I27" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="J27" s="5" t="n">
-        <v>-0.0463</v>
+      <c r="J27" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>0.0083</v>
-      </c>
-      <c r="L27" s="7" t="n">
-        <v>0.0376</v>
-      </c>
-      <c r="M27" s="10" t="n">
-        <v>0</v>
-      </c>
+        <v>0.059</v>
+      </c>
+      <c r="L27" s="5" t="n">
+        <v>-0.0122</v>
+      </c>
+      <c r="M27" s="5" t="n">
+        <v>-0.0494</v>
+      </c>
+      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
-        </is>
-      </c>
-      <c r="B28" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>-0.079</v>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>0.0501</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>0.1244</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>-0.0239</v>
+        <v>-0.0063</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>-0.2176</v>
+        <v>-0.1361</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>-0.0619</v>
-      </c>
-      <c r="G28" s="5" t="n">
-        <v>-0.0398</v>
+        <v>-0.0924</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>0.0591</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>-0.0501</v>
+        <v>-0.1014</v>
       </c>
       <c r="I28" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="J28" s="7" t="n">
-        <v>0.0926</v>
-      </c>
-      <c r="K28" s="5" t="n">
-        <v>-0.1354</v>
+      <c r="J28" s="5" t="n">
+        <v>-0.0463</v>
+      </c>
+      <c r="K28" s="7" t="n">
+        <v>0.0083</v>
       </c>
       <c r="L28" s="7" t="n">
-        <v>0.0428</v>
+        <v>0.0376</v>
       </c>
       <c r="M28" s="10" t="n">
         <v>0</v>
       </c>
+      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="n">
-        <v>0.0998</v>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>-0.0337</v>
-      </c>
-      <c r="D29" s="7" t="n">
-        <v>0.0309</v>
-      </c>
-      <c r="E29" s="7" t="n">
-        <v>0.1633</v>
-      </c>
-      <c r="F29" s="7" t="n">
-        <v>0.0555</v>
+        <v>-0.079</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>-0.0239</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>-0.2176</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>-0.0619</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>-0.0136</v>
-      </c>
-      <c r="H29" s="7" t="n">
-        <v>0.0502</v>
-      </c>
-      <c r="I29" s="7" t="n">
-        <v>0.0983</v>
+        <v>-0.0398</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>-0.0501</v>
+      </c>
+      <c r="I29" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0922</v>
+        <v>0.0926</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>-0.0548</v>
-      </c>
-      <c r="L29" s="5" t="n">
-        <v>-0.0204</v>
-      </c>
-      <c r="M29" s="7" t="n">
-        <v>0.0983</v>
-      </c>
+        <v>-0.1354</v>
+      </c>
+      <c r="L29" s="7" t="n">
+        <v>0.0428</v>
+      </c>
+      <c r="M29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="n">
-        <v>0</v>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>0.0998</v>
       </c>
       <c r="C30" s="5" t="n">
-        <v>-0.0497</v>
-      </c>
-      <c r="D30" s="5" t="n">
-        <v>-0.0049</v>
+        <v>-0.0337</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>0.0309</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>0.2184</v>
-      </c>
-      <c r="F30" s="5" t="n">
-        <v>-0.0022</v>
+        <v>0.1633</v>
+      </c>
+      <c r="F30" s="7" t="n">
+        <v>0.0555</v>
       </c>
       <c r="G30" s="5" t="n">
-        <v>-0.101</v>
-      </c>
-      <c r="H30" s="5" t="n">
-        <v>-0.1513</v>
+        <v>-0.0136</v>
+      </c>
+      <c r="H30" s="7" t="n">
+        <v>0.0502</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>0.0494</v>
+        <v>0.0983</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>0.0464</v>
-      </c>
-      <c r="K30" s="7" t="n">
-        <v>0.0837</v>
+        <v>0.0922</v>
+      </c>
+      <c r="K30" s="5" t="n">
+        <v>-0.0548</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>-0.0285</v>
+        <v>-0.0204</v>
       </c>
       <c r="M30" s="7" t="n">
-        <v>0.0494</v>
-      </c>
+        <v>0.0983</v>
+      </c>
+      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="n">
-        <v>0.0452</v>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>-0.1072</v>
+        <v>-0.0497</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>-0.073</v>
-      </c>
-      <c r="E31" s="5" t="n">
-        <v>-0.2179</v>
+        <v>-0.0049</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>0.2184</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>-0.07389999999999999</v>
+        <v>-0.0022</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>-0.09180000000000001</v>
+        <v>-0.101</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>-0.2111</v>
-      </c>
-      <c r="I31" s="5" t="n">
-        <v>-0.1968</v>
+        <v>-0.1513</v>
+      </c>
+      <c r="I31" s="7" t="n">
+        <v>0.0494</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.0232</v>
-      </c>
-      <c r="K31" s="5" t="n">
-        <v>-0.0992</v>
+        <v>0.0464</v>
+      </c>
+      <c r="K31" s="7" t="n">
+        <v>0.0837</v>
       </c>
       <c r="L31" s="5" t="n">
-        <v>-0.126</v>
-      </c>
-      <c r="M31" s="5" t="n">
-        <v>-0.123</v>
-      </c>
+        <v>-0.0285</v>
+      </c>
+      <c r="M31" s="7" t="n">
+        <v>0.0494</v>
+      </c>
+      <c r="N31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>0.0497</v>
-      </c>
-      <c r="C32" s="7" t="n">
-        <v>0.1696</v>
-      </c>
-      <c r="D32" s="7" t="n">
-        <v>0.197</v>
-      </c>
-      <c r="E32" s="7" t="n">
-        <v>0.1088</v>
-      </c>
-      <c r="F32" s="7" t="n">
-        <v>0.1949</v>
-      </c>
-      <c r="G32" s="7" t="n">
-        <v>0.1067</v>
-      </c>
-      <c r="H32" s="7" t="n">
-        <v>0.1001</v>
-      </c>
-      <c r="I32" s="7" t="n">
-        <v>0.2949</v>
-      </c>
-      <c r="J32" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" s="7" t="n">
-        <v>0.0207</v>
-      </c>
-      <c r="L32" s="7" t="n">
-        <v>0.1822</v>
-      </c>
-      <c r="M32" s="7" t="n">
-        <v>0.0979</v>
-      </c>
+        <v>0.0452</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>-0.1072</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>-0.073</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>-0.2179</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>-0.07389999999999999</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>-0.09180000000000001</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>-0.2111</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>-0.1968</v>
+      </c>
+      <c r="J32" s="7" t="n">
+        <v>0.0232</v>
+      </c>
+      <c r="K32" s="5" t="n">
+        <v>-0.0992</v>
+      </c>
+      <c r="L32" s="5" t="n">
+        <v>-0.126</v>
+      </c>
+      <c r="M32" s="5" t="n">
+        <v>-0.123</v>
+      </c>
+      <c r="N32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>0.0502</v>
-      </c>
-      <c r="C33" s="5" t="n">
-        <v>-0.07190000000000001</v>
-      </c>
-      <c r="D33" s="5" t="n">
-        <v>-0.038</v>
+        <v>0.0497</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>0.1696</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>0.197</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.1912</v>
+        <v>0.1088</v>
       </c>
       <c r="F33" s="7" t="n">
-        <v>0.0414</v>
-      </c>
-      <c r="G33" s="5" t="n">
-        <v>-0.0556</v>
+        <v>0.1949</v>
+      </c>
+      <c r="G33" s="7" t="n">
+        <v>0.1067</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.0506</v>
-      </c>
-      <c r="I33" s="5" t="n">
-        <v>-0.0495</v>
-      </c>
-      <c r="J33" s="7" t="n">
-        <v>0.0459</v>
-      </c>
-      <c r="K33" s="5" t="n">
-        <v>-0.0341</v>
-      </c>
-      <c r="L33" s="5" t="n">
-        <v>-0.0326</v>
+        <v>0.1001</v>
+      </c>
+      <c r="I33" s="7" t="n">
+        <v>0.2949</v>
+      </c>
+      <c r="J33" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="7" t="n">
+        <v>0.0207</v>
+      </c>
+      <c r="L33" s="7" t="n">
+        <v>0.1822</v>
       </c>
       <c r="M33" s="7" t="n">
-        <v>0.1961</v>
-      </c>
+        <v>0.0979</v>
+      </c>
+      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C34" s="7" t="n">
-        <v>0.1493</v>
-      </c>
-      <c r="D34" s="7" t="n">
-        <v>0.1437</v>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>0.0502</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>-0.07190000000000001</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>-0.038</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>0.2521</v>
+        <v>0.1912</v>
       </c>
       <c r="F34" s="7" t="n">
-        <v>0.1167</v>
-      </c>
-      <c r="G34" s="7" t="n">
-        <v>0.067</v>
+        <v>0.0414</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>-0.0556</v>
       </c>
       <c r="H34" s="7" t="n">
-        <v>0.2012</v>
-      </c>
-      <c r="I34" s="7" t="n">
-        <v>0.1476</v>
+        <v>0.0506</v>
+      </c>
+      <c r="I34" s="5" t="n">
+        <v>-0.0495</v>
       </c>
       <c r="J34" s="7" t="n">
-        <v>0.2307</v>
-      </c>
-      <c r="K34" s="7" t="n">
-        <v>0.1137</v>
-      </c>
-      <c r="L34" s="7" t="n">
-        <v>0.0896</v>
+        <v>0.0459</v>
+      </c>
+      <c r="K34" s="5" t="n">
+        <v>-0.0341</v>
+      </c>
+      <c r="L34" s="5" t="n">
+        <v>-0.0326</v>
       </c>
       <c r="M34" s="7" t="n">
-        <v>0.0982</v>
-      </c>
+        <v>0.1961</v>
+      </c>
+      <c r="N34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="n">
-        <v>0.0498</v>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>0.1067</v>
+        <v>0.1493</v>
       </c>
       <c r="D35" s="7" t="n">
+        <v>0.1437</v>
+      </c>
+      <c r="E35" s="7" t="n">
+        <v>0.2521</v>
+      </c>
+      <c r="F35" s="7" t="n">
+        <v>0.1167</v>
+      </c>
+      <c r="G35" s="7" t="n">
         <v>0.067</v>
       </c>
-      <c r="E35" s="5" t="n">
-        <v>-0.3813</v>
-      </c>
-      <c r="F35" s="7" t="n">
-        <v>0.2229</v>
-      </c>
-      <c r="G35" s="7" t="n">
-        <v>0.166</v>
-      </c>
       <c r="H35" s="7" t="n">
-        <v>0.6077</v>
+        <v>0.2012</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1478</v>
-      </c>
-      <c r="J35" s="5" t="n">
-        <v>-0.046</v>
+        <v>0.1476</v>
+      </c>
+      <c r="J35" s="7" t="n">
+        <v>0.2307</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>0.0569</v>
+        <v>0.1137</v>
       </c>
       <c r="L35" s="7" t="n">
-        <v>0.1336</v>
-      </c>
-      <c r="M35" s="5" t="n">
-        <v>-0.0491</v>
-      </c>
+        <v>0.0896</v>
+      </c>
+      <c r="M35" s="7" t="n">
+        <v>0.0982</v>
+      </c>
+      <c r="N35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="n">
-        <v>-0.1496</v>
-      </c>
-      <c r="C36" s="5" t="n">
-        <v>-0.2555</v>
-      </c>
-      <c r="D36" s="5" t="n">
-        <v>-0.1632</v>
-      </c>
-      <c r="E36" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" s="5" t="n">
-        <v>-0.3853</v>
-      </c>
-      <c r="G36" s="5" t="n">
-        <v>-0.2642</v>
-      </c>
-      <c r="H36" s="5" t="n">
-        <v>-1.2007</v>
-      </c>
-      <c r="I36" s="5" t="n">
-        <v>-0.1965</v>
-      </c>
-      <c r="J36" s="7" t="n">
-        <v>0.046</v>
-      </c>
-      <c r="K36" s="5" t="n">
-        <v>-0.1745</v>
-      </c>
-      <c r="L36" s="5" t="n">
-        <v>-0.2249</v>
-      </c>
-      <c r="M36" t="inlineStr"/>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>0.1067</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>-0.3813</v>
+      </c>
+      <c r="F36" s="7" t="n">
+        <v>0.2229</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <v>0.166</v>
+      </c>
+      <c r="H36" s="7" t="n">
+        <v>0.6077</v>
+      </c>
+      <c r="I36" s="7" t="n">
+        <v>0.1478</v>
+      </c>
+      <c r="J36" s="5" t="n">
+        <v>-0.046</v>
+      </c>
+      <c r="K36" s="7" t="n">
+        <v>0.0569</v>
+      </c>
+      <c r="L36" s="7" t="n">
+        <v>0.1336</v>
+      </c>
+      <c r="M36" s="5" t="n">
+        <v>-0.0491</v>
+      </c>
+      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
-        </is>
-      </c>
-      <c r="B37" s="10" t="n">
-        <v>0</v>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>-0.1496</v>
       </c>
       <c r="C37" s="5" t="n">
-        <v>-0.0355</v>
+        <v>-0.2555</v>
       </c>
       <c r="D37" s="5" t="n">
-        <v>-0.0295</v>
-      </c>
-      <c r="E37" s="5" t="n">
-        <v>-0.2712</v>
+        <v>-0.1632</v>
+      </c>
+      <c r="E37" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>-0.1066</v>
+        <v>-0.3853</v>
       </c>
       <c r="G37" s="5" t="n">
-        <v>-0.0215</v>
-      </c>
-      <c r="H37" s="7" t="n">
-        <v>0.5536</v>
+        <v>-0.2642</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>-1.2007</v>
       </c>
       <c r="I37" s="5" t="n">
-        <v>-0.0984</v>
-      </c>
-      <c r="J37" s="5" t="n">
-        <v>-0.1379</v>
-      </c>
-      <c r="K37" s="7" t="n">
-        <v>0.0527</v>
+        <v>-0.1965</v>
+      </c>
+      <c r="J37" s="7" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="K37" s="5" t="n">
+        <v>-0.1745</v>
       </c>
       <c r="L37" s="5" t="n">
-        <v>-0.0478</v>
+        <v>-0.2249</v>
       </c>
       <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B38" s="10" t="n">
         <v>0</v>
       </c>
       <c r="C38" s="5" t="n">
-        <v>-0.06469999999999999</v>
+        <v>-0.0355</v>
       </c>
       <c r="D38" s="5" t="n">
-        <v>-0.07870000000000001</v>
-      </c>
-      <c r="E38" s="7" t="n">
-        <v>0.2176</v>
+        <v>-0.0295</v>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>-0.2712</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>-0.1542</v>
+        <v>-0.1066</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>-0.1268</v>
-      </c>
-      <c r="H38" s="5" t="n">
-        <v>-0.2511</v>
+        <v>-0.0215</v>
+      </c>
+      <c r="H38" s="7" t="n">
+        <v>0.5536</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>-0.0978</v>
+        <v>-0.0984</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>-0.0464</v>
+        <v>-0.1379</v>
       </c>
       <c r="K38" s="7" t="n">
-        <v>0.07240000000000001</v>
+        <v>0.0527</v>
       </c>
       <c r="L38" s="5" t="n">
-        <v>-0.06610000000000001</v>
+        <v>-0.0478</v>
       </c>
       <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="n">
-        <v>0.0497</v>
-      </c>
-      <c r="C39" s="7" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="D39" s="7" t="n">
-        <v>0.0746</v>
-      </c>
-      <c r="E39" s="5" t="n">
-        <v>-0.1632</v>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>-0.06469999999999999</v>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>-0.07870000000000001</v>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>0.2176</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>-0.0293</v>
-      </c>
-      <c r="G39" s="7" t="n">
-        <v>0.026</v>
+        <v>-0.1542</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>-0.1268</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>-0.1503</v>
-      </c>
-      <c r="I39" s="7" t="n">
-        <v>0.2457</v>
-      </c>
-      <c r="J39" s="7" t="n">
-        <v>0.0925</v>
+        <v>-0.2511</v>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>-0.0978</v>
+      </c>
+      <c r="J39" s="5" t="n">
+        <v>-0.0464</v>
       </c>
       <c r="K39" s="7" t="n">
         <v>0.07240000000000001</v>
       </c>
-      <c r="L39" s="7" t="n">
-        <v>0.057</v>
+      <c r="L39" s="5" t="n">
+        <v>-0.06610000000000001</v>
       </c>
       <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>0.0502</v>
+        <v>0.0497</v>
       </c>
       <c r="C40" s="7" t="n">
-        <v>0.07630000000000001</v>
+        <v>0.023</v>
       </c>
       <c r="D40" s="7" t="n">
-        <v>0.1465</v>
-      </c>
-      <c r="E40" s="7" t="n">
-        <v>0.0546</v>
-      </c>
-      <c r="F40" s="7" t="n">
-        <v>0.1337</v>
+        <v>0.0746</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>-0.1632</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>-0.0293</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="H40" s="7" t="n">
-        <v>0.2513</v>
+        <v>0.026</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>-0.1503</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>0.1975</v>
+        <v>0.2457</v>
       </c>
       <c r="J40" s="7" t="n">
-        <v>0.231</v>
+        <v>0.0925</v>
       </c>
       <c r="K40" s="7" t="n">
-        <v>0.0311</v>
+        <v>0.07240000000000001</v>
       </c>
       <c r="L40" s="7" t="n">
-        <v>0.1375</v>
+        <v>0.057</v>
       </c>
       <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="n">
+        <v>0.0502</v>
+      </c>
+      <c r="C41" s="7" t="n">
+        <v>0.07630000000000001</v>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>0.1465</v>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>0.0546</v>
+      </c>
+      <c r="F41" s="7" t="n">
+        <v>0.1337</v>
+      </c>
+      <c r="G41" s="7" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H41" s="7" t="n">
+        <v>0.2513</v>
+      </c>
+      <c r="I41" s="7" t="n">
+        <v>0.1975</v>
+      </c>
+      <c r="J41" s="7" t="n">
+        <v>0.231</v>
+      </c>
+      <c r="K41" s="7" t="n">
+        <v>0.0311</v>
+      </c>
+      <c r="L41" s="7" t="n">
+        <v>0.1375</v>
+      </c>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>2026-01-13</t>
         </is>
       </c>
-      <c r="B41" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C41" s="7" t="n">
+      <c r="B42" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="7" t="n">
         <v>0.0319</v>
       </c>
-      <c r="D41" s="7" t="n">
+      <c r="D42" s="7" t="n">
         <v>0.0056</v>
       </c>
-      <c r="E41" s="7" t="n">
+      <c r="E42" s="7" t="n">
         <v>0.2997</v>
       </c>
-      <c r="F41" s="5" t="n">
+      <c r="F42" s="5" t="n">
         <v>-0.0684</v>
       </c>
-      <c r="G41" s="7" t="n">
+      <c r="G42" s="7" t="n">
         <v>0.09420000000000001</v>
       </c>
-      <c r="H41" s="7" t="n">
+      <c r="H42" s="7" t="n">
         <v>0.2515</v>
       </c>
-      <c r="I41" s="5" t="n">
+      <c r="I42" s="5" t="n">
         <v>-0.0496</v>
       </c>
-      <c r="J41" s="5" t="n">
+      <c r="J42" s="5" t="n">
         <v>-0.0461</v>
       </c>
-      <c r="K41" s="7" t="n">
+      <c r="K42" s="7" t="n">
         <v>0.0964</v>
       </c>
-      <c r="L41" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M41" t="inlineStr"/>
+      <c r="L42" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>